<commit_message>
Insumos perecibles de Gastronomia, sub-ubicaciones reales, fix rename Modulo
Importa 852 insumos del catalogo de Gastronomia (lista de insumos
gastronomia.xlsx) reusando los campos perecibles ya existentes en
Articulo de Inventario, que ahora se muestran segun es_perecible en
cualquier modulo (antes ocultos fijo). Agrega las 8 sub-ubicaciones reales
de Gastronomia (Cocina I/II, Pasteleria, Almacen, etc, leidas de las hojas
de 20.GASTRONOMIA.xlsx) y actualiza UBICACIONES.xlsx con la revision
completa de ubicaciones del CEDHI. Elimina 21.BAÑOS DE GASTRONOMIA.xlsx
(duplicado exacto de 2 hojas ya presentes en 20.GASTRONOMIA.xlsx) y la
plantilla suelta sin uso real.

Corrige Modulo.before_rename/after_rename para que el Role "Admin
{modulo}" se renombre junto con el Modulo (antes quedaba con el nombre
viejo, desincronizado de rol_admin).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos_iniciales/lista de insumos gastronomia.xlsx
+++ b/datos_iniciales/lista de insumos gastronomia.xlsx
@@ -4278,47 +4278,47 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4330,35 +4330,35 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4366,7 +4366,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4374,7 +4374,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4382,19 +4382,19 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4402,23 +4402,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -4426,15 +4426,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4442,7 +4442,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4450,15 +4450,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4470,7 +4470,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4478,7 +4478,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4486,19 +4486,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4510,23 +4510,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -4534,19 +4534,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4562,7 +4562,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4574,11 +4574,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4902,10 +4902,10 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="B1:T883"/>
-  <sheetFormatPr defaultColWidth="11.4453125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="19.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.34"/>

</xml_diff>